<commit_message>
Auto update Pengadaan 2026-10-22 08:09:07
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-22).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-22).xlsx
@@ -1012,27 +1012,35 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
-        <v>1</v>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
-        <v>1</v>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="10" t="n">
-        <v>1796500000</v>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1154,27 +1162,35 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>3</v>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E20" s="7" t="n">
-        <v>3</v>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G20" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>3839600910</v>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
@@ -1300,13 +1316,13 @@
         <v>93</v>
       </c>
       <c r="D23" s="10" t="n">
-        <v>1148350728</v>
+        <v>1145584728</v>
       </c>
       <c r="E23" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F23" s="10" t="n">
-        <v>62227794</v>
+        <v>59461794</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>5</v>
@@ -1331,22 +1347,22 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>403884747</v>
+        <v>414639535</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>74152766</v>
+        <v>84907554</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>128214258</v>
+        <v>78869208</v>
       </c>
       <c r="I24" s="7" t="n">
         <v>62</v>
@@ -1365,22 +1381,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>147</v>
+        <v>122</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>972358399</v>
+        <v>963345953</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>146596290</v>
+        <v>137583844</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>1345382085</v>
+        <v>116218702</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>109</v>
@@ -1399,22 +1415,22 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D26" s="9" t="n">
         <v>497942073</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F26" s="9" t="n">
         <v>338217900</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>3037348900</v>
+        <v>338050900</v>
       </c>
       <c r="I26" s="7" t="n">
         <v>22</v>
@@ -1470,13 +1486,13 @@
         <v>100</v>
       </c>
       <c r="D28" s="9" t="n">
-        <v>890948817</v>
+        <v>900575817</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>28881000</v>
+        <v>38508000</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>1</v>
@@ -1504,13 +1520,13 @@
         <v>181</v>
       </c>
       <c r="D29" s="10" t="n">
-        <v>2532439288</v>
+        <v>2541943441</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>58</v>
       </c>
       <c r="F29" s="10" t="n">
-        <v>1219004247</v>
+        <v>1228508400</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>58</v>
@@ -1535,22 +1551,22 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>367878502</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>80601092</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>227435607</v>
+        <v>77435607</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>48</v>
@@ -1572,13 +1588,13 @@
         <v>52</v>
       </c>
       <c r="D31" s="10" t="n">
-        <v>283157746</v>
+        <v>283301771</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F31" s="10" t="n">
-        <v>30118025</v>
+        <v>30262050</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>5</v>
@@ -1606,13 +1622,13 @@
         <v>122</v>
       </c>
       <c r="D32" s="9" t="n">
-        <v>764274671</v>
+        <v>767894130</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>6</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>103722907</v>
+        <v>107342366</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>6</v>
@@ -1640,13 +1656,13 @@
         <v>44</v>
       </c>
       <c r="D33" s="10" t="n">
-        <v>278301799</v>
+        <v>366634933</v>
       </c>
       <c r="E33" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F33" s="10" t="n">
-        <v>20641550</v>
+        <v>108974684</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>5</v>
@@ -1708,13 +1724,13 @@
         <v>66</v>
       </c>
       <c r="D35" s="10" t="n">
-        <v>463836830</v>
+        <v>463972148</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F35" s="10" t="n">
-        <v>93231105</v>
+        <v>93366423</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>6</v>
@@ -1742,13 +1758,13 @@
         <v>76</v>
       </c>
       <c r="D36" s="9" t="n">
-        <v>761250273</v>
+        <v>761771973</v>
       </c>
       <c r="E36" s="7" t="n">
         <v>13</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>333822118</v>
+        <v>334343818</v>
       </c>
       <c r="G36" s="7" t="n">
         <v>13</v>
@@ -1773,22 +1789,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>854862891</v>
+        <v>1235454791</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>81094602</v>
+        <v>461686502</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>1530548790</v>
+        <v>451166160</v>
       </c>
       <c r="I37" s="4" t="n">
         <v>85</v>
@@ -1810,13 +1826,13 @@
         <v>97</v>
       </c>
       <c r="D38" s="9" t="n">
-        <v>382731831</v>
+        <v>384332451</v>
       </c>
       <c r="E38" s="7" t="n">
         <v>12</v>
       </c>
       <c r="F38" s="9" t="n">
-        <v>100392718</v>
+        <v>101993338</v>
       </c>
       <c r="G38" s="7" t="n">
         <v>12</v>
@@ -1841,22 +1857,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>1312371275</v>
+        <v>1337901275</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>353323156</v>
+        <v>378853156</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>415595436</v>
+        <v>375518886</v>
       </c>
       <c r="I39" s="4" t="n">
         <v>92</v>
@@ -1980,13 +1996,13 @@
         <v>50</v>
       </c>
       <c r="D43" s="10" t="n">
-        <v>727698127</v>
+        <v>708077545</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F43" s="10" t="n">
-        <v>54570486</v>
+        <v>34949904</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>3</v>
@@ -2011,22 +2027,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>151137140</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>83626512</v>
+        <v>72726534</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>15</v>
@@ -2095,22 +2111,22 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>1167699071</v>
+        <v>1119046661</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>173625311</v>
+        <v>124972901</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>318350703</v>
+        <v>121983128</v>
       </c>
       <c r="I46" s="7" t="n">
         <v>167</v>
@@ -2216,13 +2232,13 @@
         <v>102</v>
       </c>
       <c r="D49" s="10" t="n">
-        <v>606361476</v>
+        <v>608286476</v>
       </c>
       <c r="E49" s="4" t="n">
         <v>15</v>
       </c>
       <c r="F49" s="10" t="n">
-        <v>203015123</v>
+        <v>204940123</v>
       </c>
       <c r="G49" s="4" t="n">
         <v>15</v>
@@ -2331,24 +2347,30 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D52" s="9" t="n">
         <v>111669795</v>
       </c>
-      <c r="E52" s="7" t="n">
-        <v>3</v>
+      <c r="E52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H52" s="9" t="n">
-        <v>68020787</v>
+      <c r="G52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I52" s="7" t="n">
         <v>14</v>
@@ -3118,13 +3140,13 @@
         <v>41</v>
       </c>
       <c r="D71" s="10" t="n">
-        <v>323431257</v>
+        <v>330321582</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F71" s="10" t="n">
-        <v>28826575</v>
+        <v>35716900</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>2</v>
@@ -3149,22 +3171,22 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D72" s="9" t="n">
         <v>637283463</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F72" s="9" t="n">
         <v>108000000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>2359971000</v>
+        <v>158730000</v>
       </c>
       <c r="I72" s="7" t="n">
         <v>29</v>
@@ -3270,7 +3292,7 @@
         <v>113</v>
       </c>
       <c r="D75" s="10" t="n">
-        <v>1398754546</v>
+        <v>1433154546</v>
       </c>
       <c r="E75" s="4" t="n">
         <v>18</v>
@@ -3288,7 +3310,7 @@
         <v>95</v>
       </c>
       <c r="J75" s="10" t="n">
-        <v>978880360</v>
+        <v>1013280360</v>
       </c>
     </row>
     <row r="76" ht="45" customHeight="1">
@@ -3304,13 +3326,13 @@
         <v>145</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>1484655470</v>
+        <v>1492289470</v>
       </c>
       <c r="E76" s="7" t="n">
         <v>24</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>200351114</v>
+        <v>207985114</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>24</v>
@@ -3333,28 +3355,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>4057</v>
+        <v>4007</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>34178424269</v>
+        <v>34679584253</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>479</v>
+        <v>429</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6397505298</v>
+        <v>6864265282</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>479</v>
+        <v>429</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>19816314757.6</v>
+        <v>6456418894.6</v>
       </c>
       <c r="I77" s="12" t="n">
         <v>3578</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>27780918971</v>
+        <v>27815318971</v>
       </c>
     </row>
   </sheetData>
@@ -3775,13 +3797,13 @@
         <v>5</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>413165330</v>
+        <v>428765330</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>261110330</v>
+        <v>276710330</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>3</v>
@@ -4211,29 +4233,45 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="10" t="n">
-        <v>199078500</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="10" t="n">
-        <v>199078500</v>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="10" t="n">
-        <v>199078500</v>
-      </c>
-      <c r="I19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="10" t="n">
-        <v>199078500</v>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -4265,45 +4303,29 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>112000000</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>112000000</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>111200910</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>111200910</v>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
@@ -4526,50 +4548,34 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>268961631</v>
-      </c>
-      <c r="E24" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F24" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G24" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H24" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I24" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J24" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K24" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L24" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>323734637</v>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>54773006</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="9" t="n">
+        <v>49345050</v>
+      </c>
+      <c r="I24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" s="9" t="n">
+        <v>49345050</v>
+      </c>
+      <c r="K24" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L24" s="9" t="n">
+        <v>49345050</v>
       </c>
       <c r="M24" s="7" t="n">
         <v>3</v>
@@ -4588,28 +4594,28 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>1590551832</v>
+        <v>1848714675</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>967379695</v>
+        <v>1225542538</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>852531955</v>
+        <v>896262562</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J25" s="10" t="n">
-        <v>852531955</v>
+        <v>896262562</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>4</v>
@@ -4834,28 +4840,28 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" s="9" t="n">
-        <v>388286000</v>
+        <v>538286000</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>138750000</v>
+        <v>288750000</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>138306000</v>
+        <v>288306000</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>138306000</v>
+        <v>288306000</v>
       </c>
       <c r="K30" s="11" t="inlineStr">
         <is>
@@ -4887,13 +4893,13 @@
         <v>7</v>
       </c>
       <c r="D31" s="10" t="n">
-        <v>490395090</v>
+        <v>477133090</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="10" t="n">
-        <v>79572000</v>
+        <v>66310000</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>1</v>
@@ -5087,13 +5093,13 @@
         <v>13</v>
       </c>
       <c r="D35" s="10" t="n">
-        <v>1667542131</v>
+        <v>1694840343</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>7</v>
       </c>
       <c r="F35" s="10" t="n">
-        <v>885723156</v>
+        <v>913021368</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>7</v>
@@ -5137,13 +5143,13 @@
         <v>39</v>
       </c>
       <c r="D36" s="9" t="n">
-        <v>5043896732</v>
+        <v>5044312982</v>
       </c>
       <c r="E36" s="7" t="n">
         <v>36</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>4775292407</v>
+        <v>4775708657</v>
       </c>
       <c r="G36" s="7" t="n">
         <v>36</v>
@@ -5184,34 +5190,34 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>2771677052</v>
+        <v>3419825552</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>1376941951</v>
+        <v>2025090451</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>1333233523</v>
+        <v>1975819523</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>1123727573</v>
+        <v>1581713573</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L37" s="10" t="n">
-        <v>366519983</v>
+        <v>713727983</v>
       </c>
       <c r="M37" s="4" t="n">
         <v>14</v>
@@ -5292,28 +5298,28 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>4127193593</v>
+        <v>4380291888</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>2421286291</v>
+        <v>2674384586</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>2388524693</v>
+        <v>2613571243</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>1346924693</v>
+        <v>1531894693</v>
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
@@ -5570,28 +5576,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>523391100</v>
+        <v>595373450</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>345935300</v>
+        <v>417917650</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>187868022</v>
+        <v>198768000</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>187868022</v>
+        <v>198768000</v>
       </c>
       <c r="K44" s="7" t="n">
         <v>2</v>
@@ -5686,28 +5692,28 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>716222170</v>
+        <v>932380105</v>
       </c>
       <c r="E46" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>471330601</v>
+      </c>
+      <c r="G46" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H46" s="9" t="n">
+        <v>448555830</v>
+      </c>
+      <c r="I46" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="F46" s="9" t="n">
-        <v>255172666</v>
-      </c>
-      <c r="G46" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H46" s="9" t="n">
-        <v>252188255</v>
-      </c>
-      <c r="I46" s="7" t="n">
-        <v>2</v>
-      </c>
       <c r="J46" s="9" t="n">
-        <v>113248255</v>
+        <v>309615830</v>
       </c>
       <c r="K46" s="11" t="inlineStr">
         <is>
@@ -6030,40 +6036,28 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D52" s="9" t="n">
-        <v>319983894</v>
-      </c>
-      <c r="E52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>660566066</v>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" s="9" t="n">
+        <v>340582172</v>
+      </c>
+      <c r="G52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>68020787</v>
+      </c>
+      <c r="I52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="J52" s="9" t="n">
+        <v>68020787</v>
       </c>
       <c r="K52" s="11" t="inlineStr">
         <is>
@@ -7215,13 +7209,13 @@
         <v>3</v>
       </c>
       <c r="D71" s="10" t="n">
-        <v>392285593</v>
+        <v>423288615</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F71" s="10" t="n">
-        <v>115814581</v>
+        <v>146817603</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>1</v>
@@ -7482,28 +7476,28 @@
         </is>
       </c>
       <c r="C76" s="7" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>3551653729</v>
+        <v>3401653729</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>714698247</v>
+        <v>564698247</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H76" s="9" t="n">
-        <v>701504825</v>
+        <v>552004825</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J76" s="9" t="n">
-        <v>701504825</v>
+        <v>552004825</v>
       </c>
       <c r="K76" s="11" t="inlineStr">
         <is>
@@ -7530,34 +7524,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>881</v>
+        <v>899</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>104567673594</v>
+        <v>106384555679</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>502</v>
+        <v>520</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>63858372291</v>
+        <v>65675254376</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>502</v>
+        <v>520</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>62925649660.41</v>
+        <v>64074268617.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>324</v>
+        <v>340</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>41497444466.02</v>
+        <v>42421386873.02</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>1117114678</v>
+        <v>1513667728</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>379</v>
@@ -8365,28 +8359,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>25286544212</v>
+        <v>26735477939</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F17" s="10" t="n">
-        <v>25286544212</v>
+        <v>26735477939</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>24845621741</v>
+        <v>26642121741</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>24845621741</v>
+        <v>26642121741</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8472,45 +8466,29 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>201600000</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>201600000</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>199078500</v>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -8542,45 +8520,29 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>1090890000</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>1090890000</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>1081900000</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>1081900000</v>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
@@ -8616,13 +8578,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="10" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8670,7 +8632,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="9" t="n">
-        <v>272000000</v>
+        <v>277500000</v>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
@@ -8716,7 +8678,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="9" t="n">
-        <v>272000000</v>
+        <v>277500000</v>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
@@ -8849,40 +8811,40 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>6905020356</v>
+        <v>49096492181</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>5361245056</v>
+        <v>47632716881</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="J25" s="10" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="L25" s="10" t="n">
-        <v>1854621974</v>
+        <v>2945468782</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N25" s="10" t="n">
-        <v>1543775300</v>
+        <v>1463775300</v>
       </c>
     </row>
     <row r="26" ht="45" customHeight="1">
@@ -9533,38 +9495,34 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>4892340896</v>
+        <v>5765940896</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>2073094000</v>
+        <v>2946694000</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>2073094000</v>
+        <v>2509890630</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>2073094000</v>
-      </c>
-      <c r="K37" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L37" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2509890630</v>
+      </c>
+      <c r="K37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L37" s="10" t="n">
+        <v>436796630</v>
       </c>
       <c r="M37" s="4" t="n">
         <v>4</v>
@@ -9653,28 +9611,28 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>3962367980</v>
+        <v>3813601480</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>3162607980</v>
+        <v>3013841480</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>2481708818</v>
+        <v>2296738818</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>2481708818</v>
+        <v>2296738818</v>
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
@@ -9880,13 +9838,13 @@
         <v>1</v>
       </c>
       <c r="D43" s="10" t="n">
-        <v>328338000</v>
+        <v>346000000</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="10" t="n">
-        <v>328338000</v>
+        <v>346000000</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
@@ -11807,28 +11765,28 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D72" s="9" t="n">
-        <v>7792798637</v>
+        <v>14398798637</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F72" s="9" t="n">
-        <v>1448692000</v>
+        <v>8054692000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>607099212</v>
+        <v>2808340212</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J72" s="9" t="n">
-        <v>607099212</v>
+        <v>2808340212</v>
       </c>
       <c r="K72" s="7" t="n">
         <v>2</v>
@@ -12019,28 +11977,28 @@
         </is>
       </c>
       <c r="C76" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>6783067600</v>
+        <v>7133067600</v>
       </c>
       <c r="E76" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F76" s="9" t="n">
+        <v>3294207800</v>
+      </c>
+      <c r="G76" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H76" s="9" t="n">
+        <v>2207941500</v>
+      </c>
+      <c r="I76" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="F76" s="9" t="n">
-        <v>2944207800</v>
-      </c>
-      <c r="G76" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H76" s="9" t="n">
-        <v>2058441500</v>
-      </c>
-      <c r="I76" s="7" t="n">
-        <v>3</v>
-      </c>
       <c r="J76" s="9" t="n">
-        <v>2058441500</v>
+        <v>2207941500</v>
       </c>
       <c r="K76" s="11" t="inlineStr">
         <is>
@@ -12067,40 +12025,40 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>217</v>
+        <v>247</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>132492199021</v>
+        <v>185764047258</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>92433332881</v>
+        <v>145779681118</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>64168731899.01</v>
+        <v>71034210805.01001</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>116</v>
+        <v>146</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>60280592799</v>
+        <v>67146071705</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>2478343628</v>
+        <v>4005987066</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>86</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>40058866140</v>
+        <v>39984366140</v>
       </c>
     </row>
   </sheetData>
@@ -13089,13 +13047,13 @@
         <v>1</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>4988300000</v>
+        <v>5040000000</v>
       </c>
       <c r="E19" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="10" t="n">
-        <v>4988300000</v>
+        <v>5040000000</v>
       </c>
       <c r="G19" s="4" t="n">
         <v>1</v>
@@ -13139,45 +13097,29 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>2688000000</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>2688000000</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>2646500000</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>2646500000</v>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
@@ -13560,40 +13502,28 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>5399320575</v>
+      </c>
+      <c r="E26" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="9" t="n">
-        <v>2699320575</v>
-      </c>
-      <c r="E26" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F26" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G26" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H26" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I26" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J26" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="F26" s="9" t="n">
+        <v>2700000000</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>2699298000</v>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="9" t="n">
+        <v>2699298000</v>
       </c>
       <c r="K26" s="11" t="inlineStr">
         <is>
@@ -17036,28 +16966,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>273281535553</v>
+        <v>278721235553</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>141675670800</v>
+        <v>147115370800</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>65889582008.97</v>
+        <v>71235380008.97</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>65889582008.97</v>
+        <v>71235380008.97</v>
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Auto update Pengadaan 2026-10-22 12:09:46
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-22).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-22).xlsx
@@ -1012,35 +1012,27 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>1796500000</v>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1162,35 +1154,27 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C20" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E20" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="F20" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G20" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>3839600910</v>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
@@ -1316,13 +1300,13 @@
         <v>93</v>
       </c>
       <c r="D23" s="10" t="n">
-        <v>1145584728</v>
+        <v>1148350728</v>
       </c>
       <c r="E23" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F23" s="10" t="n">
-        <v>59461794</v>
+        <v>62227794</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>5</v>
@@ -1347,22 +1331,22 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>414639535</v>
+        <v>403884747</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F24" s="9" t="n">
-        <v>84907554</v>
+        <v>74152766</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H24" s="9" t="n">
-        <v>78869208</v>
+        <v>128214258</v>
       </c>
       <c r="I24" s="7" t="n">
         <v>62</v>
@@ -1381,22 +1365,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>122</v>
+        <v>147</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>963345953</v>
+        <v>972358399</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>137583844</v>
+        <v>146596290</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>116218702</v>
+        <v>1345382085</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>109</v>
@@ -1415,22 +1399,22 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D26" s="9" t="n">
         <v>497942073</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F26" s="9" t="n">
         <v>338217900</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>338050900</v>
+        <v>3037348900</v>
       </c>
       <c r="I26" s="7" t="n">
         <v>22</v>
@@ -1486,13 +1470,13 @@
         <v>100</v>
       </c>
       <c r="D28" s="9" t="n">
-        <v>900575817</v>
+        <v>890948817</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="9" t="n">
-        <v>38508000</v>
+        <v>28881000</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>1</v>
@@ -1520,13 +1504,13 @@
         <v>181</v>
       </c>
       <c r="D29" s="10" t="n">
-        <v>2541943441</v>
+        <v>2532439288</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>58</v>
       </c>
       <c r="F29" s="10" t="n">
-        <v>1228508400</v>
+        <v>1219004247</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>58</v>
@@ -1551,22 +1535,22 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>367878502</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>80601092</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>77435607</v>
+        <v>227435607</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>48</v>
@@ -1588,13 +1572,13 @@
         <v>52</v>
       </c>
       <c r="D31" s="10" t="n">
-        <v>283301771</v>
+        <v>283157746</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F31" s="10" t="n">
-        <v>30262050</v>
+        <v>30118025</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>5</v>
@@ -1622,13 +1606,13 @@
         <v>122</v>
       </c>
       <c r="D32" s="9" t="n">
-        <v>767894130</v>
+        <v>764274671</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>6</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>107342366</v>
+        <v>103722907</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>6</v>
@@ -1656,13 +1640,13 @@
         <v>44</v>
       </c>
       <c r="D33" s="10" t="n">
-        <v>366634933</v>
+        <v>278301799</v>
       </c>
       <c r="E33" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F33" s="10" t="n">
-        <v>108974684</v>
+        <v>20641550</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>5</v>
@@ -1724,13 +1708,13 @@
         <v>66</v>
       </c>
       <c r="D35" s="10" t="n">
-        <v>463972148</v>
+        <v>463836830</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F35" s="10" t="n">
-        <v>93366423</v>
+        <v>93231105</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>6</v>
@@ -1758,13 +1742,13 @@
         <v>76</v>
       </c>
       <c r="D36" s="9" t="n">
-        <v>761771973</v>
+        <v>761250273</v>
       </c>
       <c r="E36" s="7" t="n">
         <v>13</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>334343818</v>
+        <v>333822118</v>
       </c>
       <c r="G36" s="7" t="n">
         <v>13</v>
@@ -1789,22 +1773,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>1235454791</v>
+        <v>854862891</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>461686502</v>
+        <v>81094602</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>451166160</v>
+        <v>1530548790</v>
       </c>
       <c r="I37" s="4" t="n">
         <v>85</v>
@@ -1826,13 +1810,13 @@
         <v>97</v>
       </c>
       <c r="D38" s="9" t="n">
-        <v>384332451</v>
+        <v>382731831</v>
       </c>
       <c r="E38" s="7" t="n">
         <v>12</v>
       </c>
       <c r="F38" s="9" t="n">
-        <v>101993338</v>
+        <v>100392718</v>
       </c>
       <c r="G38" s="7" t="n">
         <v>12</v>
@@ -1857,22 +1841,22 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>1337901275</v>
+        <v>1312371275</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>378853156</v>
+        <v>353323156</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>375518886</v>
+        <v>415595436</v>
       </c>
       <c r="I39" s="4" t="n">
         <v>92</v>
@@ -1996,13 +1980,13 @@
         <v>50</v>
       </c>
       <c r="D43" s="10" t="n">
-        <v>708077545</v>
+        <v>727698127</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F43" s="10" t="n">
-        <v>34949904</v>
+        <v>54570486</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>3</v>
@@ -2027,22 +2011,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>151137140</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>72726534</v>
+        <v>83626512</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>15</v>
@@ -2111,22 +2095,22 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>1119046661</v>
+        <v>1167699071</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>124972901</v>
+        <v>173625311</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>121983128</v>
+        <v>318350703</v>
       </c>
       <c r="I46" s="7" t="n">
         <v>167</v>
@@ -2232,13 +2216,13 @@
         <v>102</v>
       </c>
       <c r="D49" s="10" t="n">
-        <v>608286476</v>
+        <v>606361476</v>
       </c>
       <c r="E49" s="4" t="n">
         <v>15</v>
       </c>
       <c r="F49" s="10" t="n">
-        <v>204940123</v>
+        <v>203015123</v>
       </c>
       <c r="G49" s="4" t="n">
         <v>15</v>
@@ -2347,30 +2331,24 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D52" s="9" t="n">
         <v>111669795</v>
       </c>
-      <c r="E52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E52" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H52" s="11" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>68020787</v>
       </c>
       <c r="I52" s="7" t="n">
         <v>14</v>
@@ -3140,13 +3118,13 @@
         <v>41</v>
       </c>
       <c r="D71" s="10" t="n">
-        <v>330321582</v>
+        <v>323431257</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F71" s="10" t="n">
-        <v>35716900</v>
+        <v>28826575</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>2</v>
@@ -3171,22 +3149,22 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D72" s="9" t="n">
         <v>637283463</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F72" s="9" t="n">
         <v>108000000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>158730000</v>
+        <v>2359971000</v>
       </c>
       <c r="I72" s="7" t="n">
         <v>29</v>
@@ -3292,7 +3270,7 @@
         <v>113</v>
       </c>
       <c r="D75" s="10" t="n">
-        <v>1433154546</v>
+        <v>1398754546</v>
       </c>
       <c r="E75" s="4" t="n">
         <v>18</v>
@@ -3310,7 +3288,7 @@
         <v>95</v>
       </c>
       <c r="J75" s="10" t="n">
-        <v>1013280360</v>
+        <v>978880360</v>
       </c>
     </row>
     <row r="76" ht="45" customHeight="1">
@@ -3326,13 +3304,13 @@
         <v>145</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>1492289470</v>
+        <v>1484655470</v>
       </c>
       <c r="E76" s="7" t="n">
         <v>24</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>207985114</v>
+        <v>200351114</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>24</v>
@@ -3355,28 +3333,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>4007</v>
+        <v>4057</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>34679584253</v>
+        <v>34178424269</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>429</v>
+        <v>479</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6864265282</v>
+        <v>6397505298</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>429</v>
+        <v>479</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>6456418894.6</v>
+        <v>19816314757.6</v>
       </c>
       <c r="I77" s="12" t="n">
         <v>3578</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>27815318971</v>
+        <v>27780918971</v>
       </c>
     </row>
   </sheetData>
@@ -3797,13 +3775,13 @@
         <v>5</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>428765330</v>
+        <v>413165330</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>276710330</v>
+        <v>261110330</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>3</v>
@@ -4233,45 +4211,29 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="10" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="10" t="n">
+        <v>199078500</v>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -4303,29 +4265,45 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>112000000</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>112000000</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>111200910</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>111200910</v>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
@@ -4548,34 +4526,50 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D24" s="9" t="n">
-        <v>323734637</v>
-      </c>
-      <c r="E24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="9" t="n">
-        <v>54773006</v>
-      </c>
-      <c r="G24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="9" t="n">
-        <v>49345050</v>
-      </c>
-      <c r="I24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="9" t="n">
-        <v>49345050</v>
-      </c>
-      <c r="K24" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L24" s="9" t="n">
-        <v>49345050</v>
+        <v>268961631</v>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L24" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M24" s="7" t="n">
         <v>3</v>
@@ -4594,28 +4588,28 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>1848714675</v>
+        <v>1590551832</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>1225542538</v>
+        <v>967379695</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>896262562</v>
+        <v>852531955</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J25" s="10" t="n">
-        <v>896262562</v>
+        <v>852531955</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>4</v>
@@ -4840,28 +4834,28 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" s="9" t="n">
-        <v>538286000</v>
+        <v>388286000</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>288750000</v>
+        <v>138750000</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="K30" s="11" t="inlineStr">
         <is>
@@ -4893,13 +4887,13 @@
         <v>7</v>
       </c>
       <c r="D31" s="10" t="n">
-        <v>477133090</v>
+        <v>490395090</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="10" t="n">
-        <v>66310000</v>
+        <v>79572000</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>1</v>
@@ -5093,13 +5087,13 @@
         <v>13</v>
       </c>
       <c r="D35" s="10" t="n">
-        <v>1694840343</v>
+        <v>1667542131</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>7</v>
       </c>
       <c r="F35" s="10" t="n">
-        <v>913021368</v>
+        <v>885723156</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>7</v>
@@ -5143,13 +5137,13 @@
         <v>39</v>
       </c>
       <c r="D36" s="9" t="n">
-        <v>5044312982</v>
+        <v>5043896732</v>
       </c>
       <c r="E36" s="7" t="n">
         <v>36</v>
       </c>
       <c r="F36" s="9" t="n">
-        <v>4775708657</v>
+        <v>4775292407</v>
       </c>
       <c r="G36" s="7" t="n">
         <v>36</v>
@@ -5190,34 +5184,34 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>3419825552</v>
+        <v>2771677052</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>2025090451</v>
+        <v>1376941951</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>1975819523</v>
+        <v>1333233523</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>1581713573</v>
+        <v>1123727573</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="L37" s="10" t="n">
-        <v>713727983</v>
+        <v>366519983</v>
       </c>
       <c r="M37" s="4" t="n">
         <v>14</v>
@@ -5298,28 +5292,28 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>4380291888</v>
+        <v>4127193593</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>2674384586</v>
+        <v>2421286291</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>2613571243</v>
+        <v>2388524693</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>1531894693</v>
+        <v>1346924693</v>
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
@@ -5576,28 +5570,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>595373450</v>
+        <v>523391100</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>417917650</v>
+        <v>345935300</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="K44" s="7" t="n">
         <v>2</v>
@@ -5692,28 +5686,28 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>932380105</v>
+        <v>716222170</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>471330601</v>
+        <v>255172666</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>448555830</v>
+        <v>252188255</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J46" s="9" t="n">
-        <v>309615830</v>
+        <v>113248255</v>
       </c>
       <c r="K46" s="11" t="inlineStr">
         <is>
@@ -6036,28 +6030,40 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D52" s="9" t="n">
-        <v>660566066</v>
-      </c>
-      <c r="E52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F52" s="9" t="n">
-        <v>340582172</v>
-      </c>
-      <c r="G52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H52" s="9" t="n">
-        <v>68020787</v>
-      </c>
-      <c r="I52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="J52" s="9" t="n">
-        <v>68020787</v>
+        <v>319983894</v>
+      </c>
+      <c r="E52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J52" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K52" s="11" t="inlineStr">
         <is>
@@ -7209,13 +7215,13 @@
         <v>3</v>
       </c>
       <c r="D71" s="10" t="n">
-        <v>423288615</v>
+        <v>392285593</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F71" s="10" t="n">
-        <v>146817603</v>
+        <v>115814581</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>1</v>
@@ -7476,28 +7482,28 @@
         </is>
       </c>
       <c r="C76" s="7" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>3401653729</v>
+        <v>3551653729</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>564698247</v>
+        <v>714698247</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H76" s="9" t="n">
-        <v>552004825</v>
+        <v>701504825</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J76" s="9" t="n">
-        <v>552004825</v>
+        <v>701504825</v>
       </c>
       <c r="K76" s="11" t="inlineStr">
         <is>
@@ -7524,34 +7530,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>899</v>
+        <v>881</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>106384555679</v>
+        <v>104567673594</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>520</v>
+        <v>502</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>65675254376</v>
+        <v>63858372291</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>520</v>
+        <v>502</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>64074268617.41</v>
+        <v>62925649660.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>340</v>
+        <v>324</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>42421386873.02</v>
+        <v>41497444466.02</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>1513667728</v>
+        <v>1117114678</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>379</v>
@@ -8359,28 +8365,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F17" s="10" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>26642121741</v>
+        <v>24845621741</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J17" s="10" t="n">
-        <v>26642121741</v>
+        <v>24845621741</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8466,29 +8472,45 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="10" t="n">
-        <v>201600000</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="10" t="n">
-        <v>201600000</v>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="10" t="n">
-        <v>199078500</v>
-      </c>
-      <c r="I19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="10" t="n">
-        <v>199078500</v>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -8520,29 +8542,45 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>1090890000</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>1090890000</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>1081900000</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>1081900000</v>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
@@ -8578,13 +8616,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="10" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8632,7 +8670,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="9" t="n">
-        <v>277500000</v>
+        <v>272000000</v>
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
@@ -8678,7 +8716,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="9" t="n">
-        <v>277500000</v>
+        <v>272000000</v>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
@@ -8811,40 +8849,40 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>49096492181</v>
+        <v>6905020356</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="F25" s="10" t="n">
-        <v>47632716881</v>
+        <v>5361245056</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>4157004750</v>
+        <v>2971571974</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="J25" s="10" t="n">
-        <v>4157004750</v>
+        <v>2971571974</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="L25" s="10" t="n">
-        <v>2945468782</v>
+        <v>1854621974</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>4</v>
       </c>
       <c r="N25" s="10" t="n">
-        <v>1463775300</v>
+        <v>1543775300</v>
       </c>
     </row>
     <row r="26" ht="45" customHeight="1">
@@ -9495,34 +9533,38 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>5765940896</v>
+        <v>4892340896</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F37" s="10" t="n">
-        <v>2946694000</v>
+        <v>2073094000</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>2509890630</v>
+        <v>2073094000</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J37" s="10" t="n">
-        <v>2509890630</v>
-      </c>
-      <c r="K37" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L37" s="10" t="n">
-        <v>436796630</v>
+        <v>2073094000</v>
+      </c>
+      <c r="K37" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M37" s="4" t="n">
         <v>4</v>
@@ -9611,28 +9653,28 @@
         </is>
       </c>
       <c r="C39" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>3813601480</v>
+        <v>3962367980</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>3013841480</v>
+        <v>3162607980</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>2296738818</v>
+        <v>2481708818</v>
       </c>
       <c r="I39" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J39" s="10" t="n">
-        <v>2296738818</v>
+        <v>2481708818</v>
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
@@ -9838,13 +9880,13 @@
         <v>1</v>
       </c>
       <c r="D43" s="10" t="n">
-        <v>346000000</v>
+        <v>328338000</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="10" t="n">
-        <v>346000000</v>
+        <v>328338000</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
@@ -11765,28 +11807,28 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D72" s="9" t="n">
-        <v>14398798637</v>
+        <v>7792798637</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F72" s="9" t="n">
-        <v>8054692000</v>
+        <v>1448692000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>2808340212</v>
+        <v>607099212</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J72" s="9" t="n">
-        <v>2808340212</v>
+        <v>607099212</v>
       </c>
       <c r="K72" s="7" t="n">
         <v>2</v>
@@ -11977,28 +12019,28 @@
         </is>
       </c>
       <c r="C76" s="7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>7133067600</v>
+        <v>6783067600</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>3294207800</v>
+        <v>2944207800</v>
       </c>
       <c r="G76" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H76" s="9" t="n">
-        <v>2207941500</v>
+        <v>2058441500</v>
       </c>
       <c r="I76" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J76" s="9" t="n">
-        <v>2207941500</v>
+        <v>2058441500</v>
       </c>
       <c r="K76" s="11" t="inlineStr">
         <is>
@@ -12025,40 +12067,40 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>247</v>
+        <v>217</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>185764047258</v>
+        <v>132492199021</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>161</v>
+        <v>131</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>145779681118</v>
+        <v>92433332881</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>161</v>
+        <v>131</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>71034210805.01001</v>
+        <v>64168731899.01</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>146</v>
+        <v>116</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>67146071705</v>
+        <v>60280592799</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>4005987066</v>
+        <v>2478343628</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>86</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>39984366140</v>
+        <v>40058866140</v>
       </c>
     </row>
   </sheetData>
@@ -13047,13 +13089,13 @@
         <v>1</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>5040000000</v>
+        <v>4988300000</v>
       </c>
       <c r="E19" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="10" t="n">
-        <v>5040000000</v>
+        <v>4988300000</v>
       </c>
       <c r="G19" s="4" t="n">
         <v>1</v>
@@ -13097,29 +13139,45 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>2688000000</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>2688000000</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>2646500000</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>2646500000</v>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
@@ -13502,28 +13560,40 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" s="9" t="n">
-        <v>5399320575</v>
-      </c>
-      <c r="E26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="9" t="n">
-        <v>2700000000</v>
-      </c>
-      <c r="G26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H26" s="9" t="n">
-        <v>2699298000</v>
-      </c>
-      <c r="I26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J26" s="9" t="n">
-        <v>2699298000</v>
+        <v>2699320575</v>
+      </c>
+      <c r="E26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J26" s="11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K26" s="11" t="inlineStr">
         <is>
@@ -16966,28 +17036,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>278721235553</v>
+        <v>273281535553</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>147115370800</v>
+        <v>141675670800</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>71235380008.97</v>
+        <v>65889582008.97</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>71235380008.97</v>
+        <v>65889582008.97</v>
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>

</xml_diff>